<commit_message>
Fix sample-ledger.xlsx: balanced balance sheet, correct Income type, proper double-entry data
</commit_message>
<xml_diff>
--- a/public/samples/sample-ledger.xlsx
+++ b/public/samples/sample-ledger.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -464,8 +464,8 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -556,45 +556,45 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Initial deposit</t>
+          <t>Owner investment</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>5001</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2024-01-05</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>Deposit</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -604,83 +604,83 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>ATM withdrawal</t>
+          <t>Owner investment</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>-200</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Liability</t>
+          <t>Asset</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2024-01-10</t>
+          <t>2024-01-05</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Deposit</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Jane Smith</t>
+          <t>City Bank</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Loan payment</t>
+          <t>Loan proceeds</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>-500</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>15000</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>2001</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Liability</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2024-01-12</t>
+          <t>2024-01-05</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -690,55 +690,55 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Acme Corp</t>
+          <t>City Bank</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Invoice #101 payment</t>
+          <t>Loan proceeds</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>5000</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3001</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Asset</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Bill</t>
+          <t>Deposit</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -748,103 +748,103 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Office supplies</t>
+          <t>Consulting revenue</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>-150</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2650</t>
+          <t>23000</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Beta Ltd</t>
+          <t>Acme Corp</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Consulting fee</t>
+          <t>Consulting revenue</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>5650</t>
+          <t>8000</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3001</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2024-01-15</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Bill</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Beta Ltd</t>
+          <t>Rent Co</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Consulting fee</t>
+          <t>Office rent Jan</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>8650</t>
+          <t>3000</t>
         </is>
       </c>
     </row>
@@ -872,38 +872,38 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2024-01-20</t>
+          <t>2024-01-15</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>Bill</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Rent Co</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Salary advance</t>
+          <t>Office rent Jan</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>-800</t>
+          <t>-3000</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>7850</t>
+          <t>20000</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2024-01-22</t>
+          <t>2024-01-20</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -930,28 +930,28 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Rent Co</t>
+          <t>Acme Corp</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Office rent Jan</t>
+          <t>Office supplies</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>-1200</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>6650</t>
+          <t>5000</t>
         </is>
       </c>
     </row>
@@ -968,38 +968,38 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2024-01-25</t>
+          <t>2024-01-20</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>Bill</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Jane Smith</t>
+          <t>Acme Corp</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Reimbursement</t>
+          <t>Office supplies</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>-2000</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>6850</t>
+          <t>18000</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-01-25</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1026,28 +1026,28 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Jane Smith</t>
+          <t>City Bank</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Loan payment</t>
+          <t>Loan repayment</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>-500</t>
+          <t>-1000</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>6350</t>
+          <t>4000</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-01-25</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1074,28 +1074,28 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Jane Smith</t>
+          <t>City Bank</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Loan payment</t>
+          <t>Loan repayment</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>-500</t>
+          <t>-1000</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>5850</t>
+          <t>17000</t>
         </is>
       </c>
     </row>
@@ -1122,88 +1122,88 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Acme Corp</t>
+          <t>Beta Ltd</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Invoice #102 payment</t>
+          <t>Consulting fee</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>1800</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>7650</t>
+          <t>22000</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>3002</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Bill</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Acme Corp</t>
+          <t>Beta Ltd</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Stationery</t>
+          <t>Consulting fee</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>-80</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>13000</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>3001</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1213,45 +1213,45 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>Bill</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Beta Ltd</t>
+          <t>City Utils</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Retainer Feb</t>
+          <t>Utilities Feb</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>1500</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>10070</t>
+          <t>6500</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Asset</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1261,225 +1261,129 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Bill</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Beta Ltd</t>
+          <t>City Utils</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Retainer Feb</t>
+          <t>Utilities Feb</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>-1500</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>12570</t>
+          <t>20500</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>3001</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Asset</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2024-02-10</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Bill</t>
+          <t>Deposit</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Rent Co</t>
+          <t>Acme Corp</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Office rent Feb</t>
+          <t>Consulting revenue</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>-1200</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>11370</t>
+          <t>28500</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Acme Corp</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Valentine bonus</t>
+          <t>Consulting revenue</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>-300</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>11070</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>5001</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>2024-02-20</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Transfer</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>John Doe</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Capital contribution</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>16070</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Asset</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>2024-02-20</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Transfer</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>John Doe</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Capital contribution</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>21070</t>
+          <t>21000</t>
         </is>
       </c>
     </row>

</xml_diff>